<commit_message>
started on maintenance track
</commit_message>
<xml_diff>
--- a/connection_docs/Arduino_Kabelbeheer_Template.xlsx
+++ b/connection_docs/Arduino_Kabelbeheer_Template.xlsx
@@ -1,28 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\kdg\kdg-y4\fablax-exp\knex-tilt-coaster\connection_docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{150BCE52-D55D-4115-80C8-C010153299A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63684A57-1362-4383-929C-E751D0F1243A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5505" yWindow="2025" windowWidth="21600" windowHeight="11385" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="station" sheetId="2" r:id="rId1"/>
-    <sheet name="tilt_drop" sheetId="7" r:id="rId2"/>
-    <sheet name="Kast" sheetId="4" r:id="rId3"/>
+    <sheet name="maintenance" sheetId="8" r:id="rId1"/>
+    <sheet name="station" sheetId="2" r:id="rId2"/>
+    <sheet name="tilt_drop" sheetId="7" r:id="rId3"/>
+    <sheet name="Kast" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="112">
   <si>
     <t>Kabel-ID</t>
   </si>
@@ -301,6 +302,63 @@
   </si>
   <si>
     <t>mac address:</t>
+  </si>
+  <si>
+    <t>rotateBayStepper-be</t>
+  </si>
+  <si>
+    <t>rotateBayStepper-pk-we-pk</t>
+  </si>
+  <si>
+    <t>rotateBayStepper-yw</t>
+  </si>
+  <si>
+    <t>rotateBayStepper-oe-gn-oe</t>
+  </si>
+  <si>
+    <t>rotateBayStepper-rd</t>
+  </si>
+  <si>
+    <t>rotateTrackStepper-be</t>
+  </si>
+  <si>
+    <t>rotateTrackStepper-pk-we-pk</t>
+  </si>
+  <si>
+    <t>rotateTrackStepper-yw</t>
+  </si>
+  <si>
+    <t>rotateTrackStepper-oe-gn-oe</t>
+  </si>
+  <si>
+    <t>rotateTrackStepper-rd</t>
+  </si>
+  <si>
+    <t>lockServo-oe</t>
+  </si>
+  <si>
+    <t>lockServo-rd</t>
+  </si>
+  <si>
+    <t>lockServo-bn</t>
+  </si>
+  <si>
+    <t>GIOP 4</t>
+  </si>
+  <si>
+    <t>mac address ESP3/Tmaintenance</t>
+  </si>
+  <si>
+    <t>xx:xx:xx:xx</t>
+  </si>
+  <si>
+    <t>GIOP 15</t>
+  </si>
+  <si>
+    <t>GIOP 16</t>
+  </si>
+  <si>
+    <t>GIOP 17</t>
   </si>
 </sst>
 </file>
@@ -701,6 +759,353 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{838EC17A-0D5A-4B77-B63F-69875AB26128}">
+  <dimension ref="A1:L26"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="33.140625" customWidth="1"/>
+    <col min="2" max="2" width="18.5703125" customWidth="1"/>
+    <col min="3" max="6" width="20" customWidth="1"/>
+    <col min="7" max="7" width="29.5703125" customWidth="1"/>
+    <col min="8" max="8" width="18" customWidth="1"/>
+    <col min="9" max="9" width="17.5703125" customWidth="1"/>
+    <col min="10" max="10" width="20.42578125" customWidth="1"/>
+    <col min="11" max="11" width="21.85546875" customWidth="1"/>
+    <col min="12" max="12" width="27.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C2" t="s">
+        <v>40</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="H2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I2" t="s">
+        <v>46</v>
+      </c>
+      <c r="J2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" t="s">
+        <v>41</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="H3" t="s">
+        <v>28</v>
+      </c>
+      <c r="I3" t="s">
+        <v>47</v>
+      </c>
+      <c r="J3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B4" t="s">
+        <v>87</v>
+      </c>
+      <c r="C4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="H4" t="s">
+        <v>28</v>
+      </c>
+      <c r="I4" t="s">
+        <v>48</v>
+      </c>
+      <c r="J4" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A5" s="3"/>
+      <c r="G5" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="H5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I5" t="s">
+        <v>49</v>
+      </c>
+      <c r="J5" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B6" t="s">
+        <v>86</v>
+      </c>
+      <c r="C6" t="s">
+        <v>40</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="H6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="B7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" t="s">
+        <v>61</v>
+      </c>
+      <c r="G8" s="1"/>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A9" s="3"/>
+      <c r="G9" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="H9" t="s">
+        <v>28</v>
+      </c>
+      <c r="I9" t="s">
+        <v>46</v>
+      </c>
+      <c r="J9" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="B10" t="s">
+        <v>86</v>
+      </c>
+      <c r="C10" t="s">
+        <v>40</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="H10" t="s">
+        <v>28</v>
+      </c>
+      <c r="I10" t="s">
+        <v>47</v>
+      </c>
+      <c r="J10" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B11" t="s">
+        <v>14</v>
+      </c>
+      <c r="C11" t="s">
+        <v>41</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="H11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I11" t="s">
+        <v>48</v>
+      </c>
+      <c r="J11" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B12" t="s">
+        <v>88</v>
+      </c>
+      <c r="C12" t="s">
+        <v>44</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="H12" t="s">
+        <v>28</v>
+      </c>
+      <c r="I12" t="s">
+        <v>49</v>
+      </c>
+      <c r="J12" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="G13" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="H13" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="B14" t="s">
+        <v>86</v>
+      </c>
+      <c r="C14" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B15" t="s">
+        <v>14</v>
+      </c>
+      <c r="C15" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="B16" t="s">
+        <v>13</v>
+      </c>
+      <c r="C16" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B18" t="s">
+        <v>87</v>
+      </c>
+      <c r="C18" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B19" t="s">
+        <v>86</v>
+      </c>
+      <c r="C19" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="B20" t="s">
+        <v>14</v>
+      </c>
+      <c r="C20" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>107</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>108</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:L26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1026,7 +1431,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC6E52F6-C4C9-4E60-AE2A-630479BCB0E8}">
   <dimension ref="A1:L26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1321,7 +1726,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:G30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
removed credentails out repo/ added LED's
</commit_message>
<xml_diff>
--- a/connection_docs/Arduino_Kabelbeheer_Template.xlsx
+++ b/connection_docs/Arduino_Kabelbeheer_Template.xlsx
@@ -8,22 +8,23 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\kdg\kdg-y4\fablax-exp\knex-tilt-coaster\connection_docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD49A419-331B-4642-9A21-B624A91AF672}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D8407A6-4B2C-428A-9207-BC1571A17858}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-22545" yWindow="5160" windowWidth="21600" windowHeight="11295" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3120" yWindow="4185" windowWidth="21600" windowHeight="11295" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="maintenance" sheetId="8" r:id="rId1"/>
     <sheet name="station" sheetId="2" r:id="rId2"/>
     <sheet name="tilt_drop" sheetId="7" r:id="rId3"/>
-    <sheet name="Kast" sheetId="4" r:id="rId4"/>
+    <sheet name="switch_track" sheetId="9" r:id="rId4"/>
+    <sheet name="Kast" sheetId="4" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="399" uniqueCount="121">
   <si>
     <t>Kabel-ID</t>
   </si>
@@ -359,6 +360,33 @@
   </si>
   <si>
     <t>GIOP 35</t>
+  </si>
+  <si>
+    <t>360Stepper-be</t>
+  </si>
+  <si>
+    <t>360Stepper-yw</t>
+  </si>
+  <si>
+    <t>360Stepper-oe-gn-oe</t>
+  </si>
+  <si>
+    <t>360Stepper-rd</t>
+  </si>
+  <si>
+    <t>360Stepper-pk-bk-pk</t>
+  </si>
+  <si>
+    <t>motor 1</t>
+  </si>
+  <si>
+    <t>motor 2</t>
+  </si>
+  <si>
+    <t>ledExitStation</t>
+  </si>
+  <si>
+    <t>GIOP 21</t>
   </si>
 </sst>
 </file>
@@ -1420,6 +1448,39 @@
         <v>42</v>
       </c>
     </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="B22" t="s">
+        <v>15</v>
+      </c>
+      <c r="C22" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="B23" t="s">
+        <v>13</v>
+      </c>
+      <c r="C23" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="B24" t="s">
+        <v>86</v>
+      </c>
+      <c r="C24" t="s">
+        <v>41</v>
+      </c>
+    </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
         <v>90</v>
@@ -1607,11 +1668,27 @@
       <c r="C8" t="s">
         <v>43</v>
       </c>
-      <c r="G8" s="1"/>
+      <c r="G8" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="H8" t="s">
+        <v>85</v>
+      </c>
+      <c r="I8" t="s">
+        <v>87</v>
+      </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" s="3"/>
-      <c r="G9" s="1"/>
+      <c r="G9" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="H9" t="s">
+        <v>84</v>
+      </c>
+      <c r="I9" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
@@ -1623,7 +1700,15 @@
       <c r="C10" t="s">
         <v>40</v>
       </c>
-      <c r="G10" s="1"/>
+      <c r="G10" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="H10" t="s">
+        <v>14</v>
+      </c>
+      <c r="I10" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
@@ -1682,40 +1767,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="B18" t="s">
-        <v>85</v>
-      </c>
-      <c r="C18" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="B19" t="s">
-        <v>84</v>
-      </c>
-      <c r="C19" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="B20" t="s">
-        <v>14</v>
-      </c>
-      <c r="C20" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>66</v>
       </c>
@@ -1730,6 +1782,441 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1473E142-137C-4D7E-9397-929A492065BD}">
+  <dimension ref="A1:M38"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="34.7109375" customWidth="1"/>
+    <col min="2" max="2" width="11.85546875" customWidth="1"/>
+    <col min="3" max="3" width="15.85546875" customWidth="1"/>
+    <col min="4" max="4" width="18.85546875" customWidth="1"/>
+    <col min="5" max="5" width="28.5703125" customWidth="1"/>
+    <col min="8" max="8" width="42.42578125" customWidth="1"/>
+    <col min="9" max="9" width="17.28515625" customWidth="1"/>
+    <col min="11" max="11" width="18.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C2" t="s">
+        <v>40</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="I2" t="s">
+        <v>28</v>
+      </c>
+      <c r="J2" t="s">
+        <v>45</v>
+      </c>
+      <c r="K2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" t="s">
+        <v>41</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="I3" t="s">
+        <v>28</v>
+      </c>
+      <c r="J3" t="s">
+        <v>46</v>
+      </c>
+      <c r="K3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B4" t="s">
+        <v>85</v>
+      </c>
+      <c r="C4" t="s">
+        <v>88</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="I4" t="s">
+        <v>28</v>
+      </c>
+      <c r="J4" t="s">
+        <v>47</v>
+      </c>
+      <c r="K4" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A5" s="3"/>
+      <c r="H5" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="I5" t="s">
+        <v>28</v>
+      </c>
+      <c r="J5" t="s">
+        <v>48</v>
+      </c>
+      <c r="K5" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B6" t="s">
+        <v>84</v>
+      </c>
+      <c r="C6" t="s">
+        <v>40</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="I6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" t="s">
+        <v>43</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="I8" t="s">
+        <v>28</v>
+      </c>
+      <c r="J8" t="s">
+        <v>45</v>
+      </c>
+      <c r="K8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A9" s="3"/>
+      <c r="H9" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="I9" t="s">
+        <v>28</v>
+      </c>
+      <c r="J9" t="s">
+        <v>46</v>
+      </c>
+      <c r="K9" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B10" t="s">
+        <v>84</v>
+      </c>
+      <c r="C10" t="s">
+        <v>40</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="I10" t="s">
+        <v>28</v>
+      </c>
+      <c r="J10" t="s">
+        <v>47</v>
+      </c>
+      <c r="K10" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="B11" t="s">
+        <v>14</v>
+      </c>
+      <c r="C11" t="s">
+        <v>41</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="I11" t="s">
+        <v>28</v>
+      </c>
+      <c r="J11" t="s">
+        <v>48</v>
+      </c>
+      <c r="K11" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="B12" t="s">
+        <v>86</v>
+      </c>
+      <c r="C12" t="s">
+        <v>60</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="I12" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B14" t="s">
+        <v>84</v>
+      </c>
+      <c r="C14" t="s">
+        <v>40</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="I14" t="s">
+        <v>85</v>
+      </c>
+      <c r="J14" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="B15" t="s">
+        <v>14</v>
+      </c>
+      <c r="C15" t="s">
+        <v>41</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="I15" t="s">
+        <v>15</v>
+      </c>
+      <c r="J15" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B16" t="s">
+        <v>13</v>
+      </c>
+      <c r="C16" t="s">
+        <v>44</v>
+      </c>
+      <c r="H16" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="I16" t="s">
+        <v>84</v>
+      </c>
+      <c r="J16" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="B18" t="s">
+        <v>85</v>
+      </c>
+      <c r="C18" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B19" t="s">
+        <v>84</v>
+      </c>
+      <c r="C19" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B20" t="s">
+        <v>14</v>
+      </c>
+      <c r="C20" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F27" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F28" t="s">
+        <v>48</v>
+      </c>
+      <c r="G28">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F29" t="s">
+        <v>47</v>
+      </c>
+      <c r="G29">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F30" t="s">
+        <v>46</v>
+      </c>
+      <c r="G30">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F31" t="s">
+        <v>45</v>
+      </c>
+      <c r="G31">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="33" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="F33" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="35" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="F35" t="s">
+        <v>48</v>
+      </c>
+      <c r="G35">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="36" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="F36" t="s">
+        <v>47</v>
+      </c>
+      <c r="G36">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="37" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="F37" t="s">
+        <v>46</v>
+      </c>
+      <c r="G37">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="38" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="F38" t="s">
+        <v>45</v>
+      </c>
+      <c r="G38">
+        <v>14</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:G30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
added leds to tiltdrop, full auto and manual works with station and tiltdrop
</commit_message>
<xml_diff>
--- a/connection_docs/Arduino_Kabelbeheer_Template.xlsx
+++ b/connection_docs/Arduino_Kabelbeheer_Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\kdg\kdg-y4\fablax-exp\knex-tilt-coaster\connection_docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18C07C93-6FF1-4488-9354-E3647CD93A96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11581B2E-86B4-441B-8D53-CB0AF524F517}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3120" yWindow="4185" windowWidth="21600" windowHeight="11295" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="maintenance" sheetId="8" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="401" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="401" uniqueCount="132">
   <si>
     <t>Kabel-ID</t>
   </si>
@@ -393,6 +393,33 @@
   </si>
   <si>
     <t>192.168.0.51</t>
+  </si>
+  <si>
+    <t>hallSensorStationConnect-1</t>
+  </si>
+  <si>
+    <t>hallSensorStationConnect-2</t>
+  </si>
+  <si>
+    <t>hallSensorStationConnect-3</t>
+  </si>
+  <si>
+    <t>hallSensorBrakeConnect-2</t>
+  </si>
+  <si>
+    <t>white/grey</t>
+  </si>
+  <si>
+    <t>hallSensorBrakeConnect-1</t>
+  </si>
+  <si>
+    <t>hallSensorBrakeConnect-3</t>
+  </si>
+  <si>
+    <t>GIOP 25</t>
+  </si>
+  <si>
+    <t>GPIO 33</t>
   </si>
 </sst>
 </file>
@@ -1692,7 +1719,7 @@
         <v>85</v>
       </c>
       <c r="I8" t="s">
-        <v>87</v>
+        <v>131</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
@@ -1701,7 +1728,7 @@
         <v>82</v>
       </c>
       <c r="H9" t="s">
-        <v>84</v>
+        <v>15</v>
       </c>
       <c r="I9" t="s">
         <v>40</v>
@@ -1721,7 +1748,7 @@
         <v>83</v>
       </c>
       <c r="H10" t="s">
-        <v>14</v>
+        <v>84</v>
       </c>
       <c r="I10" t="s">
         <v>41</v>
@@ -1853,7 +1880,7 @@
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>69</v>
+        <v>123</v>
       </c>
       <c r="B2" t="s">
         <v>84</v>
@@ -1876,10 +1903,10 @@
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>70</v>
+        <v>124</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>86</v>
       </c>
       <c r="C3" t="s">
         <v>41</v>
@@ -1899,13 +1926,13 @@
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>71</v>
+        <v>125</v>
       </c>
       <c r="B4" t="s">
-        <v>85</v>
+        <v>13</v>
       </c>
       <c r="C4" t="s">
-        <v>88</v>
+        <v>60</v>
       </c>
       <c r="H4" s="1" t="s">
         <v>113</v>
@@ -1937,10 +1964,10 @@
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>72</v>
+        <v>128</v>
       </c>
       <c r="B6" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C6" t="s">
         <v>40</v>
@@ -1954,10 +1981,10 @@
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>74</v>
+        <v>126</v>
       </c>
       <c r="B7" t="s">
-        <v>14</v>
+        <v>86</v>
       </c>
       <c r="C7" t="s">
         <v>41</v>
@@ -1965,10 +1992,10 @@
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>73</v>
+        <v>129</v>
       </c>
       <c r="B8" t="s">
-        <v>15</v>
+        <v>127</v>
       </c>
       <c r="C8" t="s">
         <v>43</v>
@@ -2029,7 +2056,7 @@
         <v>76</v>
       </c>
       <c r="B11" t="s">
-        <v>14</v>
+        <v>86</v>
       </c>
       <c r="C11" t="s">
         <v>41</v>
@@ -2052,10 +2079,10 @@
         <v>77</v>
       </c>
       <c r="B12" t="s">
-        <v>86</v>
+        <v>13</v>
       </c>
       <c r="C12" t="s">
-        <v>60</v>
+        <v>130</v>
       </c>
       <c r="H12" s="1" t="s">
         <v>115</v>
@@ -2132,7 +2159,7 @@
         <v>85</v>
       </c>
       <c r="C18" t="s">
-        <v>87</v>
+        <v>131</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
added ledboard ESP, and basic code for displaying text per block
</commit_message>
<xml_diff>
--- a/connection_docs/Arduino_Kabelbeheer_Template.xlsx
+++ b/connection_docs/Arduino_Kabelbeheer_Template.xlsx
@@ -8,23 +8,24 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\kdg\kdg-y4\fablax-exp\knex-tilt-coaster\connection_docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4349607C-8C7E-4481-9BD8-C1FBF4F9459E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDC16591-FF91-455E-9FF3-70BDF30FB17B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="maintenance" sheetId="8" r:id="rId1"/>
     <sheet name="station" sheetId="2" r:id="rId2"/>
     <sheet name="tilt_drop" sheetId="7" r:id="rId3"/>
-    <sheet name="switch_track" sheetId="9" r:id="rId4"/>
-    <sheet name="Kast" sheetId="4" r:id="rId5"/>
+    <sheet name="brakes" sheetId="10" r:id="rId4"/>
+    <sheet name="switch_track" sheetId="9" r:id="rId5"/>
+    <sheet name="Kast" sheetId="4" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="433" uniqueCount="143">
   <si>
     <t>Kabel-ID</t>
   </si>
@@ -1889,6 +1890,139 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C48264F-142C-40E1-9C1A-0210AEF3A877}">
+  <dimension ref="A1:E20"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="34.7109375" customWidth="1"/>
+    <col min="2" max="2" width="11.85546875" customWidth="1"/>
+    <col min="3" max="3" width="15.85546875" customWidth="1"/>
+    <col min="4" max="4" width="18.85546875" customWidth="1"/>
+    <col min="5" max="5" width="28.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="B2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="B3" t="s">
+        <v>86</v>
+      </c>
+      <c r="C3" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="3"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="B6" t="s">
+        <v>85</v>
+      </c>
+      <c r="C6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="B7" t="s">
+        <v>86</v>
+      </c>
+      <c r="C7" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="B8" t="s">
+        <v>127</v>
+      </c>
+      <c r="C8" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="3"/>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="1"/>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="1"/>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="1"/>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="1"/>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="1"/>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="1"/>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" s="1"/>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" s="1"/>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1473E142-137C-4D7E-9397-929A492065BD}">
   <dimension ref="A1:M38"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2323,7 +2457,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:G30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>